<commit_message>
Trackers: Epic 11 Sprint 4 Bugs and Sprint 5 Finance delete
Founder 2026-10-22: the substantial bugs fixed along the way are a sprint of
Epic 11. Sprint 4 Bugs (NF-4.1 .. NF-4.13), 12 of 13: the client's four fixes
from the Play Store build, XCODITS QA BUG-16 / BUG-04 / BUG-14 / ACCESS-12 /
BUG-15, App Store 5.1.2 AI consent, the old Finance delete getting the books
wrong, files saving inside the app; open: WhatsApp gave no reply to a PDF.
Sprint 5 Finance delete (NF-5.1 .. NF-5.8), 8 of 8, per the epic's
one-sprint-per-client-feature rule (docs/FINANCE_DELETE_PLAN.md).
Sprints 2 and 3 carry their commits now they are pushed. Epic 11 is 48 of 53;
the Master is 947 of 1068.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic11_New_Features.xlsx
+++ b/docs/DecisionOS_Epic11_New_Features.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -498,7 +498,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -507,7 +506,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21 (Requests). Founder 2026-10-22: every new feature the client asks for is a sprint of this epic.</t>
+          <t>2026-10-21 (Requests). Founder 2026-10-22: every new feature the client asks for is a sprint of this epic, and the substantial bugs fixed along the way are Sprint 4 - Bugs.</t>
         </is>
       </c>
     </row>
@@ -519,7 +518,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Client feature requests: the Requests plan (Requests_Feature_Plan.png, decisions 2026-10-21) and FEATURE-08 Notification history (2026-10-22).</t>
+          <t>Client feature requests: the Requests plan (Requests_Feature_Plan.png, decisions 2026-10-21), FEATURE-08 Notification history and FEATURE-03 Preferred name (2026-10-22), Finance delete (2026-10-22); bugs from the client's Play Store build and the XCODITS QA report (2026-10-21).</t>
         </is>
       </c>
     </row>
@@ -535,7 +534,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -544,11 +542,10 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Sprint 1 Requests shipped (58ce262) - Phase 3 items open. Sprint 2 Notification history shipped (46bb6a0). Sprint 3 Preferred name built and checked 2026-10-22.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
+          <t>Sprint 1 Requests shipped (58ce262) - Phase 3 items open. Sprint 2 Notification history shipped (46bb6a0). Sprint 3 Preferred name shipped (6c9bdf1). Sprint 4 Bugs: 12 of 13 fixed (e46b7cc, e352141); WhatsApp no-reply open. Sprint 5 Finance delete shipped (e352141).</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -561,7 +558,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -574,7 +570,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
@@ -582,7 +577,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
@@ -638,7 +632,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
@@ -694,7 +687,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
@@ -745,6 +737,116 @@
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 4 -- Bugs</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>routers/desk.py, routers/tasks.py, hooks/useUiScale.js, services/ingestion.py, pages/Captures.js, components/mobile/Walkthrough.jsx, lib/native/files.js, services/finance_trash.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>The substantial bugs fixed along the way: the client's four from the Play Store build, the XCODITS QA bugs, App Store 5.1.2 AI consent, the old Finance delete getting the books wrong, and files that would not save inside the app. Open: WhatsApp gave no reply to a PDF on 2026-10-22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>XCODITS QA report 2026-10-21 (BUG-16, BUG-04, BUG-14, ACCESS-12, BUG-15); client fixes 1-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>In progress -- 12 of 13 Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5 -- Finance delete</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>services/finance_trash.py, routers/finance_trash.py, pages/finance/FinanceDelete.jsx, components/neuglass/DataList.jsx, pages/finance/FinanceRecords.jsx, pages/Captures.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>The client imported wrong records from Tally and could not take them out. One delete for every door that asks first, says what goes with it, keeps issued GST invoices, and can be put back for 30 days; Undo this import; select and delete; delete everything (owner, after a copy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>docs/FINANCE_DELETE_PLAN.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -761,7 +863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -783,14 +885,14 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Features the client asks for, one sprint each: plan, build, test and ship the feature as a unit.</t>
+          <t>Features the client asks for, one sprint each: plan, build, test and ship the feature as a unit. Sprint 4 collects the substantial bugs fixed along the way.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Epic 11 progress: 28 of 32 items Done  (88%).  Sprint 1 Requests (shipped 58ce262; Phase 3 open), Sprint 2 Notification history (46bb6a0), Sprint 3 Preferred name (built 2026-10-22).</t>
+          <t>Epic 11 progress: 48 of 53 items Done  (91%).  Sprint 1 Requests (shipped 58ce262; Phase 3 open), Sprint 2 Notification history (46bb6a0), Sprint 3 Preferred name (6c9bdf1), Sprint 4 Bugs (e46b7cc, e352141; WhatsApp open), Sprint 5 Finance delete (e352141).</t>
         </is>
       </c>
     </row>
@@ -927,6 +1029,72 @@
       <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Client FEATURE-03: a Preferred name in the profile, used by the greetings ('Good afternoon, Rhea', not 'S'); people who never set one are greeted by the first word of their name that is not an initial. Plan: docs/PREFERRED_NAME_PLAN.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Bugs</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>12</v>
+      </c>
+      <c r="D9" t="n">
+        <v>13</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Substantial bugs fixed along the way: the client's four fixes from the Play Store build (Delayed vs Overdue, people on a task, the Workflows tile, phone scale with a bigger font), the XCODITS QA bugs (BUG-16, BUG-04, BUG-14, ACCESS-12, BUG-15), App Store 5.1.2 AI consent, the old Finance delete, files saving inside the app. Open: WhatsApp gave no reply to a PDF (2026-10-22).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Finance delete</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Client: a wrong Tally import and no way to delete it. One delete for every door - one record, a selection, an import undone, everything - that asks first, says what goes with it, keeps issued GST invoices, and can be put back for 30 days. Plan: docs/FINANCE_DELETE_PLAN.md.</t>
         </is>
       </c>
     </row>
@@ -941,7 +1109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2075,7 +2243,7 @@
       <c r="J20" s="4" t="n"/>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/NOTIFICATION_HISTORY_PLAN.md Was NH-1.1 (briefly Epic 12).</t>
+          <t>Done 2026-10-22 - 46bb6a0. docs/NOTIFICATION_HISTORY_PLAN.md Was NH-1.1 (briefly Epic 12).</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
@@ -2131,7 +2299,7 @@
       <c r="J21" s="4" t="n"/>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/NOTIFICATION_HISTORY_PLAN.md Also fixed: the bell's 'need you' badge tested a `kind` field no notification carries, so it was always 0; the server counts the asks now (services/notifications.NEEDS_YOU_TYPES). Was NH-1.2 (briefly Epic 12).</t>
+          <t>Done 2026-10-22 - 46bb6a0. docs/NOTIFICATION_HISTORY_PLAN.md Also fixed: the bell's 'need you' badge tested a `kind` field no notification carries, so it was always 0; the server counts the asks now (services/notifications.NEEDS_YOU_TYPES). Was NH-1.2 (briefly Epic 12).</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
@@ -2187,7 +2355,7 @@
       <c r="J22" s="4" t="n"/>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/NOTIFICATION_HISTORY_PLAN.md Was NH-1.3 (briefly Epic 12).</t>
+          <t>Done 2026-10-22 - 46bb6a0. docs/NOTIFICATION_HISTORY_PLAN.md Was NH-1.3 (briefly Epic 12).</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -2243,7 +2411,7 @@
       <c r="J23" s="4" t="n"/>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/NOTIFICATION_HISTORY_PLAN.md Was NH-1.4 (briefly Epic 12).</t>
+          <t>Done 2026-10-22 - 46bb6a0. docs/NOTIFICATION_HISTORY_PLAN.md Was NH-1.4 (briefly Epic 12).</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
@@ -2299,7 +2467,7 @@
       <c r="J24" s="4" t="n"/>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/NOTIFICATION_HISTORY_PLAN.md tests/test_notification_history.py: 8 tests. Was NH-1.5 (briefly Epic 12).</t>
+          <t>Done 2026-10-22 - 46bb6a0. docs/NOTIFICATION_HISTORY_PLAN.md tests/test_notification_history.py: 8 tests. Was NH-1.5 (briefly Epic 12).</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -2355,7 +2523,7 @@
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/NOTIFICATION_HISTORY_PLAN.md Was NH-2.1 (briefly Epic 12).</t>
+          <t>Done 2026-10-22 - 46bb6a0. docs/NOTIFICATION_HISTORY_PLAN.md Was NH-2.1 (briefly Epic 12).</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -2411,7 +2579,7 @@
       <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/NOTIFICATION_HISTORY_PLAN.md Opens on the latest five with Show more, so the sections below stay in reach; links to Notifications. Was NH-2.2 (briefly Epic 12).</t>
+          <t>Done 2026-10-22 - 46bb6a0. docs/NOTIFICATION_HISTORY_PLAN.md Opens on the latest five with Show more, so the sections below stay in reach; links to Notifications. Was NH-2.2 (briefly Epic 12).</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2467,7 +2635,7 @@
       <c r="J27" s="4" t="n"/>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/NOTIFICATION_HISTORY_PLAN.md Was NH-2.3 (briefly Epic 12).</t>
+          <t>Done 2026-10-22 - 46bb6a0. docs/NOTIFICATION_HISTORY_PLAN.md Was NH-2.3 (briefly Epic 12).</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
@@ -2523,7 +2691,7 @@
       <c r="J28" s="4" t="n"/>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/NOTIFICATION_HISTORY_PLAN.md Checked as Priya on the scratch DB: badge 3 need you / 24 new; read -&gt; History with Undo; History paged to the oldest (36); Move back to New; Settings section; phone width. Was NH-2.4 (briefly Epic 12).</t>
+          <t>Done 2026-10-22 - 46bb6a0. docs/NOTIFICATION_HISTORY_PLAN.md Checked as Priya on the scratch DB: badge 3 need you / 24 new; read -&gt; History with Undo; History paged to the oldest (36); Move back to New; Settings section; phone width. Was NH-2.4 (briefly Epic 12).</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
@@ -2579,7 +2747,7 @@
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/PREFERRED_NAME_PLAN.md</t>
+          <t>Done 2026-10-22 - 6c9bdf1. docs/PREFERRED_NAME_PLAN.md</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
@@ -2635,7 +2803,7 @@
       <c r="J30" s="4" t="n"/>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/PREFERRED_NAME_PLAN.md Also skips a title (Mr, Mrs, Ms, Dr, Prof, Er, Smt) and two-or-three capitals before another word; 'S.Rhea' counts as 'S. Rhea'.</t>
+          <t>Done 2026-10-22 - 6c9bdf1. docs/PREFERRED_NAME_PLAN.md Also skips a title (Mr, Mrs, Ms, Dr, Prof, Er, Smt) and two-or-three capitals before another word; 'S.Rhea' counts as 'S. Rhea'.</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
@@ -2691,7 +2859,7 @@
       <c r="J31" s="4" t="n"/>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/PREFERRED_NAME_PLAN.md</t>
+          <t>Done 2026-10-22 - 6c9bdf1. docs/PREFERRED_NAME_PLAN.md</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
@@ -2747,7 +2915,7 @@
       <c r="J32" s="4" t="n"/>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/PREFERRED_NAME_PLAN.md</t>
+          <t>Done 2026-10-22 - 6c9bdf1. docs/PREFERRED_NAME_PLAN.md</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
@@ -2803,12 +2971,1258 @@
       <c r="J33" s="4" t="n"/>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-22 (awaiting push). docs/PREFERRED_NAME_PLAN.md tests/test_preferred_name.py: 23 tests incl. a guard that the screen-side rule matches the server's. Browser (scratch DB, 'S Rhea'): Desk 'Good morning, Rhea.' with nothing set; preferred 'Riya' -&gt; Desk, Dex welcome and Ops all say Riya; preview updates as you type.</t>
+          <t>Done 2026-10-22 - 6c9bdf1. docs/PREFERRED_NAME_PLAN.md tests/test_preferred_name.py: 23 tests incl. a guard that the screen-side rule matches the server's. Browser (scratch DB, 'S Rhea'): Desk 'Good morning, Rhea.' with nothing set; preferred 'Riya' -&gt; Desk, Dex welcome and Ops all say Riya; preview updates as you type.</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
           <t>Client FEATURE-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.1</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>routers/desk.py _delayed_count, routers/tasks.py list_tasks, pages/MyWork.js</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Desk / My Work</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Delayed tile opens the same list it counts</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Client, on the Play Store build: Desk said Delayed 18 and the Overdue list it opened was empty. The task list returned only the newest tasks, so on a company with hundreds finished the late ones fell off. The list now returns every open task plus the newest 500 finished, and the tile counts with the list's own query, in IST days.</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-21 - e46b7cc (client Fix 1).</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.2</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>services/tasks.py, lib/taskAccess.js, pages/MyWork.js, pages/Tasks.js</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Any number of people on a task, and Everyone</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>A task held at most 10 helpers. No cap now, and the people picker starts with Everyone (N) once there are two or more.</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-21 - e46b7cc (client Fix 2).</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.3</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>pages/desk/WorkflowsTile.jsx, pages/Workflows.js, index.css</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Desk / Workflows</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Workflows tile: no Approve, one Open in Workflows</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Approve left the tile (approving belongs on the card). One full-width Open in Workflows opens the board on the card's stage with the card glowing; picking another board no longer jumps back.</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr"/>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-21 - e46b7cc (client Fix 3).</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.4</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>hooks/useUiScale.js, android MainActivity.java</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Phone scale on OnePlus / OPPO / Realme (OxygenOS, ColorOS 16)</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>With the system font size above normal, the web view zoomed the text twice and the Desk broke (tiles cut off). useUiScale measures type and boxes separately; the fallback viewport sets setUseWideViewPort. Checked on a OnePlus 13s and the emulator.</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I37" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-21 - e46b7cc (client Fix 4).</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.5</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>services/ingestion.py upload_scope, routers/finance.py, pages/Captures.js, pages/finance/ReviewPanel.js</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Finance / Inbox</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>BUG-16: uploaded bills appear in Pending and Filed</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>A bill read but not filed waited nowhere, and one filed was never seen again by someone without Finance. Pending and Filed list uploads (the owner and Finance: the company's; others: their own), Discard works, and the toast says where the record went.</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr"/>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-21 - e46b7cc.</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>XCODITS QA 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.6</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>routers/tasks.py, services/recurrence.py, services/task_timing.py, pages/MyWork.js, bootstrap/lifecycle.py</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>BUG-04: how late a task was stays after it closes</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Closing from the checklist did not stamp the completion, so the lateness was lost. Overdue shows 'Overdue - N days', finished shows 'Finished N days late' or 'on time', a finished task's due date is locked until reopened, and a recurring task's next one is due today, not in the past. Migration task_completed_at_v2 backfills.</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-21 - e46b7cc.</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>XCODITS QA 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.7</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>android AndroidManifest.xml, pages/MyWork.js</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>BUG-14: camera buttons open the camera</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>On Android 11 and later the camera intent was invisible to the app (no &lt;queries&gt;), so Photo opened the gallery; picking the same photo twice did nothing.</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr"/>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-21 - e46b7cc.</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>XCODITS QA 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.8</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>components/mobile/Walkthrough.jsx</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>ACCESS-12: the walkthrough teaches only what you can do</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>It taught Decide and the books to people without them. The steps follow the person's role and permissions.</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-21 - e46b7cc.</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>XCODITS QA 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.9</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>pages/Ledger.js</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>BUG-15: the Money 'index box' button</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>An unlabelled tray icon on the phone's Quick capture card that did nothing on the Inbox. Gone (the Inbox tab carries the count), and a one-cell tab bar is no longer drawn.</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr"/>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e46b7cc, e352141.</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>XCODITS QA 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.10</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>MicDictateButton.js, useDexCapture.js, lib/aiConsent.js, pages/Settings.js</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>AI / App Store</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>App Store 5.1.2: AI consent asked first, every provider named</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Dex sent voice and text to AI providers before asking. It asks first, and names each provider.</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I43" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-21 - c6182c3.</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>App Store review</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.11</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>routers/ledger.py deletes -&gt; services/finance_trash.py</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Deleting in Finance got the books wrong</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>A deleted payment left its invoice 'received'; a deleted invoice deleted a payment split across other invoices; a deleted expense left its bill in Bills to pay and its asset behind; one tap deleted with no question, no undo and no record; deleting the latest issued invoice reissued its number; Dex kept quoting deleted records. Fixed by Sprint 5's one delete.</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I44" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.1</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141.</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.12</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>lib/native/files.js; MoneyActions, BrainDocuments, DexAnswer, Captures, RequestCard, MyWork, financeKit, ReviewPanel</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Files save inside the Android and iOS apps</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>The app's web view has no download handler: invoice PDF, Brain document and Dex export buttons did nothing, and links to bills and attachments opened a browser that was not signed in. In the app a file now goes to the share sheet (save to Files or Drive, or send on WhatsApp or mail); the web is unchanged. @capacitor/filesystem 8.1.4, @capacitor/share 8.0.3.</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I45" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141. Checked on the Android emulator; iOS has the plugins, not yet run on a device.</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Found 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>NF-4.13</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>services/whatsapp.py, integrations/whatsapp.py, routers/whatsapp.py</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>A PDF sent on WhatsApp got no reply</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-22: the client's PDF got no 'Received' reply. No inbound WhatsApp code changed since 8 Oct, so likely an expired Meta token, the sender not routed to a workspace (pending member, number in two workspaces), or the webhook not delivered. A reply Meta refuses is never logged today. Next: a read-only look at production wa_events for that number, then log Meta's refusals on each event.</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr"/>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>Investigated 2026-10-22 in code; waiting on the production check.</t>
+        </is>
+      </c>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.1</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>services/finance_trash.py, routers/finance_trash.py, routers/ledger.py</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>One delete for every door</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Plan (what goes with it, what changes on what stays) -&gt; remove (a copy in finance_trash_rows first, then put right what stays, then out of the books) -&gt; restore. Payment applications, invoice balances, a bill's expense and stock, an expense's asset, request links, standalone payments; the Brain's notes go too. The old DELETE endpoints route through it; an activity and an audit row each time.</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I47" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141. docs/FINANCE_DELETE_PLAN.md</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.2</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>pages/finance/FinanceDelete.jsx, pages/Ledger.js</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Every delete asks first, and has Undo</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>The sheet lists what it deletes, what goes with it because they belong together, and what changes on what stays; the toast after it has Undo.</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.1</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141.</t>
+        </is>
+      </c>
+      <c r="L48" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.3</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>components/neuglass/DataList.jsx, pages/finance/FinanceRecords.jsx, MoneyActions.jsx, routers/ledger.py list_payables</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Select and delete on every list</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Select, tick (cards on a phone, a column on a laptop), a bar above the dock. Supplier bills and payments made can be deleted; Payments made is listed under Expenses.</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.2</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141.</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.4</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>routers/finance_trash.py imports, services/ingestion.py, routers/finance.py, pages/Captures.js</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Finance / Inbox</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Undo this import</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>On each filed upload in Money &gt; Inbox &gt; Filed: everything the import filed goes, with the payments it matched to older invoices taken off them; contacts used elsewhere and tasks already started are kept. The card then says Undone, with Put back. Imports now stamp their id on stock and follow-up tasks; older imports are found by the moments they were filed.</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.1</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141.</t>
+        </is>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.5</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>services/finance_trash.py list_trash / restore / purge_expired, workers/schedulers.py</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Recently deleted, for 30 days</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Finance &gt; ... &gt; Recently deleted puts any delete back for 30 days; the scheduler empties older ones.</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I51" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.1</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141.</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.6</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>routers/finance_trash.py everything / export</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Delete all Finance records (owner)</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>A copy first (a one-time link to the books as a spreadsheet), then the company's name typed. Contacts, tasks and requests are not touched.</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.1</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141.</t>
+        </is>
+      </c>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.7</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>services/finance_trash.py is_issued, routers/invoicing.py _next_number</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Finance / GST</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>Issued GST invoices kept; their numbers never reissued</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Kept by default with credit-note advice; only the owner can override. A retired number, or one in Recently deleted, is skipped by the next number and refused when typed.</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I53" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.1</t>
+        </is>
+      </c>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141.</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>NF-5.8</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_finance_records_can_be_deleted_and_put_back.py, browser, Android emulator</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Tests and checks</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>11 tests on a throwaway database plus the route baseline; checked in the browser at phone size and on the Android emulator.</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr"/>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-22 - e352141.</t>
+        </is>
+      </c>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>Client 2026-10-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Trackers: Sprint 10 - onboarding, the first-week tour, Dex widget
Epic 11 gains Sprint 10 (NF-10.1 to NF-10.23), set after the Finance
periods sprint: the Dex home-screen widget and its black-window bug, the
single glowing transcribing line, signup redrawn (blueprint ground, the OS
taking shape beside every step, each interview answer naming what it
added, waits that say what is happening, interview pause, Basics in
pictures, the build carrying the canvas, the last screen's KPIs and
explorer, the team map), the circle-alignment bug, the first-week tour
inside the real desktop app and its wrong-targets bug, desktop taking
the phone's task view and card, the phone lightbox bug, a camera beside
attach, the phone's grey freeze on Decide, and release 1.1.0. Two open:
transcription mode (founder's call) and the backend deploy.

Epic 11 at 129 of 138; all epics 1028 of 1153.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic11_New_Features.xlsx
+++ b/docs/DecisionOS_Epic11_New_Features.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B68"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1086,6 +1086,61 @@
       <c r="B68" s="4" t="inlineStr">
         <is>
           <t>Done -- 7 of 7 (feature)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 10 -- Onboarding, first-week tour, Dex widget</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>pages/Signup.js, pages/onboarding/* (OsAssembly, OsMap, WaitStory, BasicsFlow, VoiceInterview, voice.js, BuildReveal, walkthrough/*), components/tour/FirstWeekTour.jsx, lib/firstTour.js, components/Layout.js, components/mobile/Walkthrough.jsx, pages/MyWork.js, pages/mywork/*, pages/desk/DeskDexWell.jsx + DexCapturePopup.jsx, components/requests/NewRequestDialog.jsx, lib/native/quick.js, index.css; android (DexWidgetProvider, DexQuickActivity, widget resources); backend services/ai/onboarding.py, routers/signup.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>The founder: onboarding is where a client is won - it must show the company being built as they answer, never leave them waiting in silence, and end with what was made and where it lives in the app; plus Dex one tap from the home screen, desktop matching the phone's task design, a camera beside attach, and the phone's grey freeze.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Founder messages and screenshots, 2026-10-29 and 2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>21 of 23 Done; open: NF-10.22 transcription mode (founder), NF-10.23 backend deploy</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1129,10 +1184,11 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Epic 11 progress: 108 of 115 items Done  (94%).  Sprint 1 Requests (shipped 58ce262; Phase 3 open), Sprint 2 Notification history (46bb6a0), Sprint 3 Preferred name (6c9bdf1), Sprint 4 Bugs (e46b7cc, e352141, delete speed; WhatsApp open), Sprint 5 Finance delete (e352141), Sprint 6 Admin console redesign (2 follow-ups open), Sprint 7 Admin console v2 (P1 1ea398d, P2 a6a8215, P3 cf8da32, P4 + P5 47e0335), Sprint 8 Phone redesign (3ecf7bf and the 2026-10-29 push), Sprint 9 Finance periods and bill review (feature).</t>
-        </is>
-      </c>
-    </row>
+          <t>Epic 11 progress: 129 of 138 items Done  (93%).  Sprint 1 Requests (shipped 58ce262; Phase 3 open), Sprint 2 Notification history (46bb6a0), Sprint 3 Preferred name (6c9bdf1), Sprint 4 Bugs (e46b7cc, e352141, delete speed; WhatsApp open), Sprint 5 Finance delete (e352141), Sprint 6 Admin console redesign (2 follow-ups open), Sprint 7 Admin console v2 (P1 1ea398d, P2 a6a8215, P3 cf8da32, P4 + P5 47e0335), Sprint 8 Phone redesign (3ecf7bf and the 2026-10-29 push), Sprint 9 Finance periods and bill review (feature), Sprint 10 Onboarding, first-week tour, Dex widget (7cc7d24 .. 8c9ae5f; 2 open).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -1464,6 +1520,39 @@
       <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Feature: Finance follows the company's financial year - opens on the FY, any quarter or half of any year, custom range, one period for Overview, Revenue and Expenses (owed money never hidden), a setting for when the year starts, rolls over by itself - and an attached bill is read first, filled in for the person to check, then saved. Plan: docs/FINANCE_PERIODS.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sprint 10</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding, first-week tour, Dex widget</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D15" t="n">
+        <v>23</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>91%</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Signup redrawn as the company's OS taking shape (blueprint ground, the OS canvas fed by every answer, waits that say what is happening, interview pause, the summary with KPIs and the What Dex built explorer); the first-week tour over the real desktop app; Dex on the Android home screen; desktop takes the phone's task view and card; a camera beside attach; the phone's grey freeze on Decide fixed; release 1.1.0. Open: transcription mode (founder's call), backend deploy.</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8107,6 +8196,1340 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.1</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>android: DexWidgetProvider.java, DexQuickActivity.java, res/layout/widget_dex.xml, res/drawable/widget_*.xml, res/xml/dex_widget_info.xml, AndroidManifest.xml, values/styles.xml; frontend/src/lib/native/quick.js, components/Layout.js, App.js (/quick)</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>Dex widget</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>Dex on the Android home screen</t>
+        </is>
+      </c>
+      <c r="F117" s="4" t="inlineStr">
+        <is>
+          <t>A home-screen widget: Ask, the app icon, Decide on a dark glass rectangle (black at ~60%, small radius). Ask and Decide open the real flows in a see-through layer over the launcher (DexQuickActivity, a translucent BridgeActivity started at /quick?mode=ask|decide; Layout draws only the dock and the tapped flow; closing returns to the home screen). The icon knob opens the app itself.</t>
+        </is>
+      </c>
+      <c r="G117" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I117" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J117" s="4" t="inlineStr"/>
+      <c r="K117" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24. Checked on the OnePlus: widget placed, Ask and Decide over the wallpaper, knob opens the app.</t>
+        </is>
+      </c>
+      <c r="L117" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.2</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>DexQuickActivity.java, AndroidManifest.xml</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="inlineStr">
+        <is>
+          <t>The widget layer opened black</t>
+        </is>
+      </c>
+      <c r="F118" s="4" t="inlineStr">
+        <is>
+          <t>On Android 17 the translucent theme alone left the window marked as covering what is under it, so the launcher stopped drawing and the clear ground showed black. The activity now asks for translucency outright (setTranslucent(true)) and drops the fixed portrait orientation that cannot coexist with it.</t>
+        </is>
+      </c>
+      <c r="G118" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H118" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I118" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J118" s="4" t="inlineStr"/>
+      <c r="K118" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24. Verified on device (occludesParent=false).</t>
+        </is>
+      </c>
+      <c r="L118" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.3</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/desk/DexCapturePopup.jsx, index.css (.ng-glow-text)</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>Dex Decide</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>One centred, glowing "Transcribing what you said" in step 1</t>
+        </is>
+      </c>
+      <c r="F119" s="4" t="inlineStr">
+        <is>
+          <t>The spinner row above the field and the pulse inside it were two loaders for one wait. Now a single line sits centred in the field and glows on a slow loop; nothing spins (held still under reduced motion).</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I119" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J119" s="4" t="inlineStr"/>
+      <c r="K119" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24. Seen on the phone.</t>
+        </is>
+      </c>
+      <c r="L119" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.4</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Signup.js, index.css (.ob-backdrop, .ob-orb)</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>Signup background: a drawn blueprint, not a photograph</t>
+        </is>
+      </c>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>A cool paper with a dot grid and two slow ink-blue and gold lights replace the signup photo, giving the glass cards their midtone; reduced motion holds it still.</t>
+        </is>
+      </c>
+      <c r="G120" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H120" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I120" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J120" s="4" t="inlineStr"/>
+      <c r="K120" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24.</t>
+        </is>
+      </c>
+      <c r="L120" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.5</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/onboarding/OsAssembly.jsx, pages/Signup.js</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>"Your OS, taking shape" beside every signup step</t>
+        </is>
+      </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>The company at the centre; pieces land round it as the founder answers - owner and team from Basics, trade, sales model and website, then the departments, workflows, approvals and rules each interview answer adds. While Dex works the hub ring turns, links carry light and a ghost slot marks the next piece. Desktop orbit (two staggered rings past six pieces, max 8 shown); phone strip, newest first.</t>
+        </is>
+      </c>
+      <c r="G121" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I121" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J121" s="4" t="inlineStr"/>
+      <c r="K121" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24; ring/label fixes 2b395c6.</t>
+        </is>
+      </c>
+      <c r="L121" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.6</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>backend: services/ai/onboarding.py (_built_pieces), routers/signup.py (/interview/answer -&gt; built)</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>Each interview answer names what it added to the OS</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>The same model call that picks the next question also returns up to three {kind, label} pieces (department, workflow, approval, task, rule, metric) from the last answer - no second request, no extra wait. Unknown kinds dropped, labels cut to 48 chars.</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H122" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I122" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J122" s="4" t="inlineStr"/>
+      <c r="K122" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24. Tests: tests/test_onboarding_builds_as_you_answer.py. Needs the Railway backend deploy to show on the live app (NF-10.23).</t>
+        </is>
+      </c>
+      <c r="L122" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.7</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/onboarding/WaitStory.jsx, VoiceInterview.js, BuildReveal.js</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Client feedback</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>Every wait says what is happening</t>
+        </is>
+      </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>Client: "the user is waiting so long with no prompt". Writing down a spoken answer, Dex choosing the next question and finding its voice, the interview warming up, the final build and the workflow layout each show a glowing line, a short story that moves on with the wait (not looping) and an easing gold line - in place of small spinners on buttons.</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I123" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J123" s="4" t="inlineStr"/>
+      <c r="K123" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24.</t>
+        </is>
+      </c>
+      <c r="L123" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.8</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/onboarding/voice.js (useAnswerRecorder), VoiceInterview.js</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>Pause and resume while answering the interview</t>
+        </is>
+      </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>While speaking, Pause/Resume sits beside Stop; resuming records into the same answer (MediaRecorder pause/resume).</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H124" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I124" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J124" s="4" t="inlineStr"/>
+      <c r="K124" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24. Not tried with a real microphone in the browser pane.</t>
+        </is>
+      </c>
+      <c r="L124" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.9</t>
+        </is>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/onboarding/BasicsFlow.js, VoiceInterview.js</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>Basics and the language pick: pictures, fewer words</t>
+        </is>
+      </c>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
+          <t>Each Basics question wears an icon tile of what it asks for instead of a step number; supporting lines cut to a few words; the language pick says one line, not two.</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I125" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J125" s="4" t="inlineStr"/>
+      <c r="K125" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24. Test pin updated (test_p2_p3_polish_batch).</t>
+        </is>
+      </c>
+      <c r="L125" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.10</t>
+        </is>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/onboarding/BuildReveal.js (building stage)</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t>The build carries the picture on</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>While Dex builds, the OS canvas keeps assembling with the interview's pieces beside the progress story, in place of a separate forge animation.</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I126" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J126" s="4" t="inlineStr"/>
+      <c r="K126" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 7cc7d24.</t>
+        </is>
+      </c>
+      <c r="L126" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.11</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/onboarding/BuildReveal.js, OsMap.jsx, walkthrough/journey.js</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="inlineStr">
+        <is>
+          <t>The last signup screen: KPIs and "What Dex built"</t>
+        </is>
+      </c>
+      <c r="F127" s="4" t="inlineStr">
+        <is>
+          <t>Counts first (teams, workflows, steps, tasks set up, sign-offs, routines - the three that wait on the workflows glow "..." until laid out), then an explorer with a tab per kind: Workflows (the route, step by step), Teams (the map), Sign-offs (gates leading to "You", removable), Routines (as My Work rows). Tell Dex and Enter unchanged.</t>
+        </is>
+      </c>
+      <c r="G127" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I127" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J127" s="4" t="inlineStr"/>
+      <c r="K127" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29/30 - 7cc7d24, f65c54a, ebb52b9. Checked on local test companies (Verma Spices, Nilgiri Leaf Co, Coastal Cashew Exports).</t>
+        </is>
+      </c>
+      <c r="L127" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.12</t>
+        </is>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/onboarding/OsMap.jsx</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>The team map: hand-offs along the ring, plain panel</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
+          <t>Teams round the company; hand-offs drawn as arcs of the ring (two-way pairs on either side), a legend under the map; a team's panel names every step of each workflow in order with its own dark, plus who it gets work from and hands work to.</t>
+        </is>
+      </c>
+      <c r="G128" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I128" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J128" s="4" t="inlineStr"/>
+      <c r="K128" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - f65c54a.</t>
+        </is>
+      </c>
+      <c r="L128" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.13</t>
+        </is>
+      </c>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/onboarding/OsMap.jsx, walkthrough/scenes.jsx</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D129" s="4" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="inlineStr">
+        <is>
+          <t>Teams and the cycle sat off their circles; the ring ran through words</t>
+        </is>
+      </c>
+      <c r="F129" s="4" t="inlineStr">
+        <is>
+          <t>An entrance's inline transform (and framer's own) replaced the centring classes, so each node sat half its size down and right of its point. Placing moved to a plain wrapper with the icon centre on the ring; names ride on white cards clear of the line.</t>
+        </is>
+      </c>
+      <c r="G129" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I129" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J129" s="4" t="inlineStr"/>
+      <c r="K129" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 - 2b395c6.</t>
+        </is>
+      </c>
+      <c r="L129" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.14</t>
+        </is>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/components/tour/FirstWeekTour.jsx, lib/firstTour.js, pages/onboarding/walkthrough/{journey.js,scenes.jsx,Player.jsx}, components/Layout.js (mount + "Take the tour")</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="inlineStr">
+        <is>
+          <t>The first-week tour, inside the real desktop app</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>Pressing Enter keeps the company's script (filled from the draft). The app plays it once, after any welcome or Terms card: their company at a glance, then spotlights on real elements - the Desk board, its numbers, the Dex well, the first workflow column, the routines bar, the My Work list, the approvals area, the Dex pill, the nav - each with a small preview in the note card filled from their company (their rule waiting, their words and the tasks Dex drafts, an order walking their workflow, a checklist ticking, the approval, Dex answering). The cycle closes it; "Start using DecisionOS" leaves the live app. Mocks only: nothing read from or written to the server. Replay from the account menu. Desktop only; the phone keeps its short walkthrough ending at the guide.</t>
+        </is>
+      </c>
+      <c r="G130" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H130" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I130" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J130" s="4" t="inlineStr"/>
+      <c r="K130" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 - 01aa146, 0f1438c. All 11 steps checked at full size on the real pages. Superseded on the way: a mock-up video walkthrough on the summary (0683789, 5e821f7, ebb52b9, a489dc9), removed.</t>
+        </is>
+      </c>
+      <c r="L130" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.15</t>
+        </is>
+      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/components/tour/FirstWeekTour.jsx</t>
+        </is>
+      </c>
+      <c r="C131" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D131" s="4" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="inlineStr">
+        <is>
+          <t>The tour pointed at the wrong things and drew its own UI</t>
+        </is>
+      </c>
+      <c r="F131" s="4" t="inlineStr">
+        <is>
+          <t>Founder: "many parts showed something else, or invented UI instead of the actual page". The Decide step looked for an element the desktop Desk does not have and fell back to the whole page, covering it with a mock; the Dex step hit a hidden duplicate test id. Targets are now measured on the real pages (desk-insight, header-scoped nav-brain), nothing is drawn over the page, and a step whose element never appears is passed over.</t>
+        </is>
+      </c>
+      <c r="G131" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H131" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I131" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J131" s="4" t="inlineStr"/>
+      <c r="K131" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 - 0f1438c.</t>
+        </is>
+      </c>
+      <c r="L131" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.16</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/MyWork.js (mobileTaskView at every width, LEGACY_TASK_BODY off)</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>Desktop parity</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>Desktop opens the phone's task view</t>
+        </is>
+      </c>
+      <c r="F132" s="4" t="inlineStr">
+        <is>
+          <t>The task drawer on desktop holds the phone's view: hero, AI Execution Guide, Steps / Documents / Activity / Notes, status at the top of Activity, the Complete / Update slider; desktop keeps manual progress % and the workflow stage on its chip. The checklist drafts itself on open at every width. The old desktop body is kept behind a flag for a week, then deleted.</t>
+        </is>
+      </c>
+      <c r="G132" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H132" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I132" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J132" s="4" t="inlineStr"/>
+      <c r="K132" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 56e7d44. Tests: My Work suite (243 passed).</t>
+        </is>
+      </c>
+      <c r="L132" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.17</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/MyWork.js (TaskCell), pages/mywork/WorkDeck.jsx (TaskSummaryCard bulk tick)</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>Desktop parity</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="inlineStr">
+        <is>
+          <t>Desktop list cards are the phone's task card</t>
+        </is>
+      </c>
+      <c r="F133" s="4" t="inlineStr">
+        <is>
+          <t>In the High / Medium / Low columns and the grid, each task is the phone's card (status, due, title, people, numbered steps, Next action, Mark as Doing / Open task) and opens the same drawer; desktop's bulk-select tick comes along.</t>
+        </is>
+      </c>
+      <c r="G133" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H133" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I133" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J133" s="4" t="inlineStr"/>
+      <c r="K133" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 56e7d44.</t>
+        </is>
+      </c>
+      <c r="L133" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.18</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/MyWork.js (lightboxDialog), pages/mywork/TaskNotes.jsx</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="inlineStr">
+        <is>
+          <t>A proof photo tapped on the phone opened nothing</t>
+        </is>
+      </c>
+      <c r="F134" s="4" t="inlineStr">
+        <is>
+          <t>The full-size photo dialog lived only in the desktop body, while the phone's attachment blocks set it. It is the view's own now, at every width. Notes say "this device", not "this phone".</t>
+        </is>
+      </c>
+      <c r="G134" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H134" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I134" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J134" s="4" t="inlineStr"/>
+      <c r="K134" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-29 - 56e7d44.</t>
+        </is>
+      </c>
+      <c r="L134" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.19</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/desk/DeskDexWell.jsx, DexCapturePopup.jsx, components/requests/NewRequestDialog.jsx</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>A camera button beside attach</t>
+        </is>
+      </c>
+      <c r="F135" s="4" t="inlineStr">
+        <is>
+          <t>Founder: "when I click attach in Dex Decide it only shows documents - I want a camera button for live shooting". Decide's "What you said" card and the new-request dialog get a camera button beside the paperclip that opens the camera straight away (capture="environment"), same upload. Ask's chat and the task view already had one.</t>
+        </is>
+      </c>
+      <c r="G135" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H135" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I135" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J135" s="4" t="inlineStr"/>
+      <c r="K135" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 - 0f1438c. In the 1.1.0 release build; not pressed in the browser pane (camera blocked there).</t>
+        </is>
+      </c>
+      <c r="L135" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.20</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>frontend/src/index.css (.ui-scale [data-dialog-overlay][data-state=closed])</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="inlineStr">
+        <is>
+          <t>The phone froze grey on Decide's "What you said"</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>Read off the device over the WebView debugger: Decide's card was open with a dialog scrim - open, taking taps - after it in &lt;body&gt; at the same z-50. The card had closed and reopened inside its wrapper's 210ms exit hold: the wrapper was reused in place while the scrim, unmounted at once on a phone, was mounted again at the end of &lt;body&gt; and painted over the card. The scrim is held for the same 210ms, so a quick close-and-reopen keeps it under its card.</t>
+        </is>
+      </c>
+      <c r="G136" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H136" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I136" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J136" s="4" t="inlineStr"/>
+      <c r="K136" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 - 8c9ae5f. Root cause confirmed on device; the fix not yet seen under the same timing.</t>
+        </is>
+      </c>
+      <c r="L136" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.21</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>android: release build (keystore.properties + release.keystore, gitignored)</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>DecisionOS 1.1.0 release build</t>
+        </is>
+      </c>
+      <c r="F137" s="4" t="inlineStr">
+        <is>
+          <t>Signed release APK, version 1.1.0 (code 11), pointing at Railway, carrying everything above. Installed on the test phone after the debug build was uninstalled (debug and release keys differ). File: Claude outputs/releases/DecisionOS-1.1.0-release-railway-2026-10-30.apk (not committed).</t>
+        </is>
+      </c>
+      <c r="G137" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H137" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I137" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J137" s="4" t="inlineStr"/>
+      <c r="K137" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30.</t>
+        </is>
+      </c>
+      <c r="L137" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.22</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>backend: integrations/stt.py (SARVAM_STT_MODEL saaras:v3, mode=translate)</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>Decide and Ask show a translation, not the words spoken</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="inlineStr">
+        <is>
+          <t>Founder saw a transcript that was not what he said. Not demo data: speech goes to Sarvam saaras:v3 in translate mode with the language auto-detected, so any language comes back as an English translation (and a noisy clip can come back invented). Founder to decide: keep translation, or switch Decide and Ask to word-for-word transcription.</t>
+        </is>
+      </c>
+      <c r="G138" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H138" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I138" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J138" s="4" t="inlineStr"/>
+      <c r="K138" s="4" t="inlineStr">
+        <is>
+          <t>Waiting on the founder's call (2026-10-30).</t>
+        </is>
+      </c>
+      <c r="L138" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.23</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>Railway backend</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="inlineStr">
+        <is>
+          <t>Deploy the backend for the interview's live pieces</t>
+        </is>
+      </c>
+      <c r="F139" s="4" t="inlineStr">
+        <is>
+          <t>NF-10.6 ships in backend/services/ai/onboarding.py and routers/signup.py; the phone and live web need it deployed to show pieces landing during the interview. Everything else in Sprint 10 works against the current server.</t>
+        </is>
+      </c>
+      <c r="G139" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H139" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I139" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J139" s="4" t="inlineStr"/>
+      <c r="K139" s="4" t="inlineStr">
+        <is>
+          <t>Needs a deploy go-ahead.</t>
+        </is>
+      </c>
+      <c r="L139" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-29/30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Trackers: Sprint 10 gains the desktop card and the Workspace
NF-10.24 to NF-10.28: the desktop task card's one steps bar (no Next
action or buttons), every card the same shape, priority as a glow along
the bottom edge, desktop My Work as the Workspace (status fence, work
tree), and the owner's team board with its per-person numbers. Sprint 10
at 26 of 28; Epic 11 at 147 of 156; all epics 1046 of 1171.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic11_New_Features.xlsx
+++ b/docs/DecisionOS_Epic11_New_Features.xlsx
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>21 of 23 Done; open: NF-10.22 transcription mode (founder), NF-10.23 backend deploy</t>
+          <t>26 of 28 Done; open: NF-10.22 transcription mode (founder), NF-10.23 backend deploy</t>
         </is>
       </c>
     </row>
@@ -1241,10 +1241,11 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Epic 11 progress: 142 of 151 items Done  (94%).  Sprint 1 Requests (shipped 58ce262; Phase 3 open), Sprint 2 Notification history (46bb6a0), Sprint 3 Preferred name (6c9bdf1), Sprint 4 Bugs (e46b7cc, e352141, delete speed; WhatsApp open), Sprint 5 Finance delete (e352141), Sprint 6 Admin console redesign (2 follow-ups open), Sprint 7 Admin console v2 (P1 1ea398d, P2 a6a8215, P3 cf8da32, P4 + P5 47e0335), Sprint 8 Phone redesign (3ecf7bf and the 2026-10-29 push), Sprint 9 Finance periods and bill review (feature), Sprint 10 Onboarding, first-week tour, Dex widget (7cc7d24 .. 8c9ae5f; 2 open), Sprint 11 Decisions to owned work (feature).</t>
-        </is>
-      </c>
-    </row>
+          <t>Epic 11 progress: 147 of 156 items Done  (94%).  Sprint 1 Requests (shipped 58ce262; Phase 3 open), Sprint 2 Notification history (46bb6a0), Sprint 3 Preferred name (6c9bdf1), Sprint 4 Bugs (e46b7cc, e352141, delete speed; WhatsApp open), Sprint 5 Finance delete (e352141), Sprint 6 Admin console redesign (2 follow-ups open), Sprint 7 Admin console v2 (P1 1ea398d, P2 a6a8215, P3 cf8da32, P4 + P5 47e0335), Sprint 8 Phone redesign (3ecf7bf and the 2026-10-29 push), Sprint 9 Finance periods and bill review (feature), Sprint 10 Onboarding, first-week tour, Dex widget (7cc7d24 .. 8c9ae5f; 2 open), Sprint 11 Decisions to owned work (feature).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -1591,14 +1592,14 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D15" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1608,7 +1609,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Signup redrawn as the company's OS taking shape (blueprint ground, the OS canvas fed by every answer, waits that say what is happening, interview pause, the summary with KPIs and the What Dex built explorer); the first-week tour over the real desktop app; Dex on the Android home screen; desktop takes the phone's task view and card; a camera beside attach; the phone's grey freeze on Decide fixed; release 1.1.0. Open: transcription mode (founder's call), backend deploy.</t>
+          <t>Signup redrawn as the company's OS taking shape (blueprint ground, the OS canvas fed by every answer, waits that say what is happening, interview pause, the summary with KPIs and the What Dex built explorer); the first-week tour over the real desktop app; Dex on the Android home screen; desktop takes the phone's task view and card; a camera beside attach; the phone's grey freeze on Decide fixed; release 1.1.0; then the desktop task card (one steps bar, every card the same shape, priority as a bottom glow) and desktop My Work as the Workspace with the owner's team board. Open: transcription mode (founder's call), backend deploy.</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L152"/>
+  <dimension ref="A1:L157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9846,35 +9847,37 @@
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>NF-11.1</t>
+          <t>NF-10.24</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t>services/task_pickup.py Company.managers / level / ladder</t>
-        </is>
-      </c>
-      <c r="C144" s="4" t="n">
-        <v>11</v>
+          <t>frontend/src/pages/mywork/WorkDeck.jsx (TaskSummaryCard desk, StepProgress), pages/MyWork.js (TaskCell)</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
         <is>
-          <t>Decisions / Team</t>
+          <t>Desktop parity</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>The team's managers, from Reports to</t>
+          <t>Desktop task card: one steps bar, no Next action or buttons</t>
         </is>
       </c>
       <c r="F144" s="4" t="inlineStr">
         <is>
-          <t>A team's managers are whoever in it reports straight to an owner (its head) or has people reporting to them (Team &gt; Reports to); their level is how far they are from the owner. No manager setting (founder: later, once a client confirms). No managers: their steps go to the owner. Two at a level: both asked.</t>
+          <t>Founder (screenshot, three areas marked): on desktop the Next action box, Mark as Doing and Open task are gone - a click anywhere on the card opens the task; the numbered step row is one bar, 'Steps n of m', that fills to match and opens the task on Steps. The tick box still only selects. The phone card is unchanged.</t>
         </is>
       </c>
       <c r="G144" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H144" s="4" t="inlineStr">
@@ -9887,10 +9890,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="J144" s="4" t="n"/>
+      <c r="J144" s="4" t="inlineStr"/>
       <c r="K144" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: heads, two heads, Priya (reports to Ravi) not a head.</t>
+          <t>Done 2026-10-30 - 4a2edc2. Checked on the local test company: card body, steps bar and tick box each do their own thing.</t>
         </is>
       </c>
       <c r="L144" s="4" t="inlineStr">
@@ -9902,40 +9905,42 @@
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>NF-11.2</t>
+          <t>NF-10.25</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>services/task_pickup.py route/place/announce; voice.build_proposal; decision_flow.approve_decision_flow; workflow_engine.on_stage_enter; routers/tasks.py create_task, reassign; routers/decisions.py add_decision_task; services/deprovisioning.py</t>
-        </is>
-      </c>
-      <c r="C145" s="4" t="n">
-        <v>11</v>
+          <t>frontend/src/pages/mywork/WorkDeck.jsx</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
         <is>
-          <t>Decisions / Work</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
-          <t>Work nobody has goes to the team's queue</t>
+          <t>Desktop task cards all the same shape</t>
         </is>
       </c>
       <c r="F145" s="4" t="inlineStr">
         <is>
-          <t>Founder: a decision makes its tasks and they land with nobody; and 'I can't say we should assign to the least number of tasks'. Now, with no person named: the team's one person; else the team's QUEUE (everyone in it sees it); high priority -&gt; the head is asked (still queued); no team or nobody in it -&gt; the owner is asked. Never by load. Same for decisions, workflow stages, New Task for a team, a task added to a decision, a task moved to another team, and someone leaving with work handed to nobody (it keeps its team now). One message per person per team.</t>
+          <t>Founder: cards uneven inside. Title and description at most two lines each, ending in '...' (full text on hover), fonts unchanged (20px / 15px); the description sits in a light glass well and 'No description' holds its place; the title, the header and the people row keep their room whether filled or not, so every card is the same height (383px across all 22 local cards) and every row lines up.</t>
         </is>
       </c>
       <c r="G145" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H145" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I145" s="11" t="inlineStr">
@@ -9943,14 +9948,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="J145" s="4" t="inlineStr">
-        <is>
-          <t>NF-11.1</t>
-        </is>
-      </c>
+      <c r="J145" s="4" t="inlineStr"/>
       <c r="K145" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: every kind of team, approval end to end (one message each, approver not told), New Task, stage, leaver, added task. Dev data: 93 of 148 open decision/workflow tasks had nobody.</t>
+          <t>Done 2026-10-30 - 4a2edc2.</t>
         </is>
       </c>
       <c r="L145" s="4" t="inlineStr">
@@ -9962,40 +9963,42 @@
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>NF-11.3</t>
+          <t>NF-10.26</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>POST /tasks/{id}/take; services/task_pickup.take; MyWork.js TakeItBar</t>
-        </is>
-      </c>
-      <c r="C146" s="4" t="n">
-        <v>11</v>
+          <t>frontend/src/pages/mywork/WorkDeck.jsx (PRIO_GLOW)</t>
+        </is>
+      </c>
+      <c r="C146" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>Take it</t>
+          <t>Priority as a glow along the card's bottom edge</t>
         </is>
       </c>
       <c r="F146" s="4" t="inlineStr">
         <is>
-          <t>Anyone in the team (or an owner) takes a queued task in one tap from the My Work drawer. One write wins; the second gets 'Priya Nair already has this task.' The head hears who took it; the decision's timeline says so.</t>
+          <t>The old desktop card's stripe came back beside the title (then shortened to the title alone), but users found it unconvincing. Priority is now a soft glow along the inside of the card's bottom edge with a 1px line - red high, orange medium, grey low - made subtler on the founder's second look. Screen readers still hear the priority.</t>
         </is>
       </c>
       <c r="G146" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H146" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I146" s="11" t="inlineStr">
@@ -10003,14 +10006,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="J146" s="4" t="inlineStr">
-        <is>
-          <t>NF-11.2</t>
-        </is>
-      </c>
+      <c r="J146" s="4" t="inlineStr"/>
       <c r="K146" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: team only, owner for no team, finished, two at once -&gt; one wins.</t>
+          <t>Done 2026-10-30 - 4a2edc2. Iterations: stripe beside title and people -&gt; title only -&gt; bottom glow -&gt; subtler glow, thinner line.</t>
         </is>
       </c>
       <c r="L146" s="4" t="inlineStr">
@@ -10022,35 +10021,37 @@
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>NF-11.4</t>
+          <t>NF-10.27</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>services/task_pickup.warn_unpicked (follow-up sweep); Settings &gt; Deadlines &gt; Work nobody has</t>
-        </is>
-      </c>
-      <c r="C147" s="4" t="n">
-        <v>11</v>
+          <t>frontend/src/pages/mywork/WorkspaceHub.jsx (StatusFence, WorkTree), pages/MyWork.js (desktop header, one scroll)</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="D147" s="4" t="inlineStr">
         <is>
-          <t>Work / Notifications</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>It keeps asking until someone has it</t>
+          <t>Desktop My Work becomes the Workspace</t>
         </is>
       </c>
       <c r="F147" s="4" t="inlineStr">
         <is>
-          <t>While a task has nobody it is asked about again, one notification per person per step however many tasks; step length is the company's own (Settings &gt; Deadlines &gt; Work nobody has). Who each step asks: NF-11.8.</t>
+          <t>Client ask via the founder. Title 'Workspace'. The Status dropdown is a fence of count tiles (All open, To do, Doing, Waiting on someone, Needs approval, Overdue, Due today, No due date, Done - '500+' where the list holds only the newest 500 finished). The switcher is a work tree: the reader's own face in the middle, My Tasks, Asked by me, All Tasks (under the owner), My requests and Approvals on branches, the path in use drawn in ink. Smart priority and + New in the header; the fence and tree scroll away with the list. Desktop only; the Approvals page keeps its room; same ?view= addresses and testids.</t>
         </is>
       </c>
       <c r="G147" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H147" s="4" t="inlineStr">
@@ -10063,14 +10064,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="J147" s="4" t="inlineStr">
-        <is>
-          <t>NF-11.2</t>
-        </is>
-      </c>
+      <c r="J147" s="4" t="inlineStr"/>
       <c r="K147" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: each step, one message for three tasks, no repeats, no head, own days.</t>
+          <t>Done 2026-10-30 - 4a2edc2. Walked as the owner (all views) and a member (own face, three branches); phone unchanged. Tests: tests/test_the_workspace_puts_the_team_first.py.</t>
         </is>
       </c>
       <c r="L147" s="4" t="inlineStr">
@@ -10082,35 +10079,37 @@
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>NF-11.5</t>
+          <t>NF-10.28</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>GET /tasks/needs-person; pages/desk/NeedsPersonSheet.jsx; Desk.js card; lib/notif.js</t>
-        </is>
-      </c>
-      <c r="C148" s="4" t="n">
-        <v>11</v>
+          <t>frontend/src/pages/mywork/WorkspaceHub.jsx (TeamBoard, personStats, PersonBar), pages/MyWork.js (boardOn, goBoard, deptBar)</t>
+        </is>
+      </c>
+      <c r="C148" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="D148" s="4" t="inlineStr">
         <is>
-          <t>Desk</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>Needs a person on the Desk</t>
+          <t>The owner's team board</t>
         </is>
       </c>
       <c r="F148" s="4" t="inlineStr">
         <is>
-          <t>Owners see every task with nobody, a head their own team's, oldest first: where it waits, how long, assign on the spot (team first) or Take it. A head may assign from their own queue. 'Assign it' notifications open the list.</t>
+          <t>The owner's desktop opens on All Tasks as a ranked board: one card per person with Open (and how many wait on someone), Overdue, Done in 30 days, On time (dated work finished by its date), a Behind / On track / Free badge, a bar of all they were given that is finished, and when work last reached them and they last finished. Rank by Delivered, On time or Overdue. The client's reference counted Total / Completed / In progress / Pending, which overlap, with a bar that did not follow from them - replaced. Team totals count tasks once. Work held by a team or nobody gets its own way in. A person opens their cards under 'Team'; Department is a segment bar here only. Counted from the list the page holds - no new endpoint.</t>
         </is>
       </c>
       <c r="G148" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H148" s="4" t="inlineStr">
@@ -10123,14 +10122,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="J148" s="4" t="inlineStr">
-        <is>
-          <t>NF-11.2</t>
-        </is>
-      </c>
+      <c r="J148" s="4" t="inlineStr"/>
       <c r="K148" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: owner / head / member scopes, head assigns, others refused.</t>
+          <t>Done 2026-10-30 - 4a2edc2.</t>
         </is>
       </c>
       <c r="L148" s="4" t="inlineStr">
@@ -10142,12 +10137,12 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>NF-11.6</t>
+          <t>NF-11.1</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>services/enrich.py goes_to; DecisionDialog.js; DexReview.jsx; decision_flow.task_assigned_line</t>
+          <t>services/task_pickup.py Company.managers / level / ladder</t>
         </is>
       </c>
       <c r="C149" s="4" t="n">
@@ -10155,22 +10150,22 @@
       </c>
       <c r="D149" s="4" t="inlineStr">
         <is>
-          <t>Decisions</t>
+          <t>Decisions / Team</t>
         </is>
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>The review says where each task will go</t>
+          <t>The team's managers, from Reports to</t>
         </is>
       </c>
       <c r="F149" s="4" t="inlineStr">
         <is>
-          <t>Before approving, each task nobody is named for says where it will wait ('Sales queue - anyone in Sales can take it', 'Karthik assigns it - high priority, Sales head', 'The owner assigns it - no team named'); the timeline after.</t>
+          <t>A team's managers are whoever in it reports straight to an owner (its head) or has people reporting to them (Team &gt; Reports to); their level is how far they are from the owner. No manager setting (founder: later, once a client confirms). No managers: their steps go to the owner. Two at a level: both asked.</t>
         </is>
       </c>
       <c r="G149" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H149" s="4" t="inlineStr">
@@ -10183,14 +10178,10 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="J149" s="4" t="inlineStr">
-        <is>
-          <t>NF-11.2</t>
-        </is>
-      </c>
+      <c r="J149" s="4" t="n"/>
       <c r="K149" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: labels and timeline lines.</t>
+          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: heads, two heads, Priya (reports to Ravi) not a head.</t>
         </is>
       </c>
       <c r="L149" s="4" t="inlineStr">
@@ -10202,12 +10193,12 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>NF-11.7</t>
+          <t>NF-11.2</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>tests/test_work_nobody_has_finds_its_person.py; docs/WORK_NOBODY_HAS.md</t>
+          <t>services/task_pickup.py route/place/announce; voice.build_proposal; decision_flow.approve_decision_flow; workflow_engine.on_stage_enter; routers/tasks.py create_task, reassign; routers/decisions.py add_decision_task; services/deprovisioning.py</t>
         </is>
       </c>
       <c r="C150" s="4" t="n">
@@ -10215,17 +10206,17 @@
       </c>
       <c r="D150" s="4" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Decisions / Work</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>Older work joins its queue; tests and browser check</t>
+          <t>Work nobody has goes to the team's queue</t>
         </is>
       </c>
       <c r="F150" s="4" t="inlineStr">
         <is>
-          <t>Tasks that already had nobody join their queue quietly; their days start then (the July backlog does not hit the owner at once) and nothing is handed out silently. Who counts as here is judged per person (NF-4.16).</t>
+          <t>Founder: a decision makes its tasks and they land with nobody; and 'I can't say we should assign to the least number of tasks'. Now, with no person named: the team's one person; else the team's QUEUE (everyone in it sees it); high priority -&gt; the head is asked (still queued); no team or nobody in it -&gt; the owner is asked. Never by load. Same for decisions, workflow stages, New Task for a team, a task added to a decision, a task moved to another team, and someone leaving with work handed to nobody (it keeps its team now). One message per person per team.</t>
         </is>
       </c>
       <c r="G150" s="4" t="inlineStr">
@@ -10235,7 +10226,7 @@
       </c>
       <c r="H150" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="I150" s="11" t="inlineStr">
@@ -10245,12 +10236,12 @@
       </c>
       <c r="J150" s="4" t="inlineStr">
         <is>
-          <t>NF-11.2</t>
+          <t>NF-11.1</t>
         </is>
       </c>
       <c r="K150" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-30 (feature). Browser, demo workspace (scratch DB) with two extra Sales people: review labels; approval placed 4 tasks (queue / head / owner / Amit the only one) and told the right people; Desk card + sheet, assigned to Divya; Priya took from the queue in My Work, head told, second take 409.</t>
+          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: every kind of team, approval end to end (one message each, approver not told), New Task, stage, leaver, added task. Dev data: 93 of 148 open decision/workflow tasks had nobody.</t>
         </is>
       </c>
       <c r="L150" s="4" t="inlineStr">
@@ -10262,12 +10253,12 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>NF-11.8</t>
+          <t>NF-11.3</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>services/task_pickup.py steps_for, warn_unpicked, needs_person, take; routers/tasks.py _heads_its_queue</t>
+          <t>POST /tasks/{id}/take; services/task_pickup.take; MyWork.js TakeItBar</t>
         </is>
       </c>
       <c r="C151" s="4" t="n">
@@ -10275,17 +10266,17 @@
       </c>
       <c r="D151" s="4" t="inlineStr">
         <is>
-          <t>Work / Notifications</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>Reminders climb the reporting tree, one level a day</t>
+          <t>Take it</t>
         </is>
       </c>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>Founder 2026-10-30: 'rather than nudging the owner with a lot of notifications' - the owner has 5 departments, each with 2 reporting, who have their own people. A task with nobody now climbs its team's reporting tree one level a day: the deepest managers first (team leads), then the next level (the head), the owner last. High priority starts at once (team leads told when it is made). Work already waiting on the owner is not chased again - it stays on the Desk. Only the step now due is asked. Every manager of the team sees and may assign its queue. Settings: one step length (pickup_step_days) instead of head/owner days.</t>
+          <t>Anyone in the team (or an owner) takes a queued task in one tap from the My Work drawer. One write wins; the second gets 'Priya Nair already has this task.' The head hears who took it; the decision's timeline says so.</t>
         </is>
       </c>
       <c r="G151" s="4" t="inlineStr">
@@ -10305,12 +10296,12 @@
       </c>
       <c r="J151" s="4" t="inlineStr">
         <is>
-          <t>NF-11.4</t>
+          <t>NF-11.2</t>
         </is>
       </c>
       <c r="K151" s="4" t="inlineStr">
         <is>
-          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: three-level Sales (leads day 1, head day 2, owner day 3, then nothing), high priority from the leads at once, any manager sees/assigns, chain that never reaches the owner. Browser: high priority went to Divya (level 2), not Karthik.</t>
+          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: team only, owner for no team, finished, two at once -&gt; one wins.</t>
         </is>
       </c>
       <c r="L151" s="4" t="inlineStr">
@@ -10322,12 +10313,12 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>NF-11.9</t>
+          <t>NF-11.4</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>services/finance_signals.py _finance_assignee, run_finance_actions</t>
+          <t>services/task_pickup.warn_unpicked (follow-up sweep); Settings &gt; Deadlines &gt; Work nobody has</t>
         </is>
       </c>
       <c r="C152" s="4" t="n">
@@ -10335,45 +10326,345 @@
       </c>
       <c r="D152" s="4" t="inlineStr">
         <is>
+          <t>Work / Notifications</t>
+        </is>
+      </c>
+      <c r="E152" s="4" t="inlineStr">
+        <is>
+          <t>It keeps asking until someone has it</t>
+        </is>
+      </c>
+      <c r="F152" s="4" t="inlineStr">
+        <is>
+          <t>While a task has nobody it is asked about again, one notification per person per step however many tasks; step length is the company's own (Settings &gt; Deadlines &gt; Work nobody has). Who each step asks: NF-11.8.</t>
+        </is>
+      </c>
+      <c r="G152" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H152" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I152" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J152" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.2</t>
+        </is>
+      </c>
+      <c r="K152" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: each step, one message for three tasks, no repeats, no head, own days.</t>
+        </is>
+      </c>
+      <c r="L152" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.5</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>GET /tasks/needs-person; pages/desk/NeedsPersonSheet.jsx; Desk.js card; lib/notif.js</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D153" s="4" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="E153" s="4" t="inlineStr">
+        <is>
+          <t>Needs a person on the Desk</t>
+        </is>
+      </c>
+      <c r="F153" s="4" t="inlineStr">
+        <is>
+          <t>Owners see every task with nobody, a head their own team's, oldest first: where it waits, how long, assign on the spot (team first) or Take it. A head may assign from their own queue. 'Assign it' notifications open the list.</t>
+        </is>
+      </c>
+      <c r="G153" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H153" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I153" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J153" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.2</t>
+        </is>
+      </c>
+      <c r="K153" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: owner / head / member scopes, head assigns, others refused.</t>
+        </is>
+      </c>
+      <c r="L153" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.6</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>services/enrich.py goes_to; DecisionDialog.js; DexReview.jsx; decision_flow.task_assigned_line</t>
+        </is>
+      </c>
+      <c r="C154" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>Decisions</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="inlineStr">
+        <is>
+          <t>The review says where each task will go</t>
+        </is>
+      </c>
+      <c r="F154" s="4" t="inlineStr">
+        <is>
+          <t>Before approving, each task nobody is named for says where it will wait ('Sales queue - anyone in Sales can take it', 'Karthik assigns it - high priority, Sales head', 'The owner assigns it - no team named'); the timeline after.</t>
+        </is>
+      </c>
+      <c r="G154" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H154" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I154" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J154" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.2</t>
+        </is>
+      </c>
+      <c r="K154" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: labels and timeline lines.</t>
+        </is>
+      </c>
+      <c r="L154" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.7</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_work_nobody_has_finds_its_person.py; docs/WORK_NOBODY_HAS.md</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D155" s="4" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="inlineStr">
+        <is>
+          <t>Older work joins its queue; tests and browser check</t>
+        </is>
+      </c>
+      <c r="F155" s="4" t="inlineStr">
+        <is>
+          <t>Tasks that already had nobody join their queue quietly; their days start then (the July backlog does not hit the owner at once) and nothing is handed out silently. Who counts as here is judged per person (NF-4.16).</t>
+        </is>
+      </c>
+      <c r="G155" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H155" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I155" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J155" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.2</t>
+        </is>
+      </c>
+      <c r="K155" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 (feature). Browser, demo workspace (scratch DB) with two extra Sales people: review labels; approval placed 4 tasks (queue / head / owner / Amit the only one) and told the right people; Desk card + sheet, assigned to Divya; Priya took from the queue in My Work, head told, second take 409.</t>
+        </is>
+      </c>
+      <c r="L155" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.8</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>services/task_pickup.py steps_for, warn_unpicked, needs_person, take; routers/tasks.py _heads_its_queue</t>
+        </is>
+      </c>
+      <c r="C156" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>Work / Notifications</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="inlineStr">
+        <is>
+          <t>Reminders climb the reporting tree, one level a day</t>
+        </is>
+      </c>
+      <c r="F156" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-30: 'rather than nudging the owner with a lot of notifications' - the owner has 5 departments, each with 2 reporting, who have their own people. A task with nobody now climbs its team's reporting tree one level a day: the deepest managers first (team leads), then the next level (the head), the owner last. High priority starts at once (team leads told when it is made). Work already waiting on the owner is not chased again - it stays on the Desk. Only the step now due is asked. Every manager of the team sees and may assign its queue. Settings: one step length (pickup_step_days) instead of head/owner days.</t>
+        </is>
+      </c>
+      <c r="G156" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H156" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I156" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J156" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.4</t>
+        </is>
+      </c>
+      <c r="K156" s="4" t="inlineStr">
+        <is>
+          <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: three-level Sales (leads day 1, head day 2, owner day 3, then nothing), high priority from the leads at once, any manager sees/assigns, chain that never reaches the owner. Browser: high priority went to Divya (level 2), not Karthik.</t>
+        </is>
+      </c>
+      <c r="L156" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-10-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>NF-11.9</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>services/finance_signals.py _finance_assignee, run_finance_actions</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
           <t>Finance / Work</t>
         </is>
       </c>
-      <c r="E152" s="4" t="inlineStr">
+      <c r="E157" s="4" t="inlineStr">
         <is>
           <t>Finance follow-ups join the Finance queue</t>
         </is>
       </c>
-      <c r="F152" s="4" t="inlineStr">
+      <c r="F157" s="4" t="inlineStr">
         <is>
           <t>Founder 2026-10-30: the automatic Finance follow-ups (chase an overdue invoice, pay a bill) went to whoever in Finance had the fewest tasks. Now they follow the same rule: Finance's one person, else the Finance queue (a chase is high priority, so Finance's nearest managers are asked at once), no Finance team -&gt; the owner; then the ladder.</t>
         </is>
       </c>
-      <c r="G152" s="4" t="inlineStr">
+      <c r="G157" s="4" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H152" s="4" t="inlineStr">
+      <c r="H157" s="4" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="I152" s="11" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="J152" s="4" t="inlineStr">
+      <c r="I157" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J157" s="4" t="inlineStr">
         <is>
           <t>NF-11.2</t>
         </is>
       </c>
-      <c r="K152" s="4" t="inlineStr">
+      <c r="K157" s="4" t="inlineStr">
         <is>
           <t>Done 2026-10-30 (feature). test_work_nobody_has_finds_its_person.py: Finance queue + manager asked, a team of one, no Finance team -&gt; owner.</t>
         </is>
       </c>
-      <c r="L152" s="4" t="inlineStr">
+      <c r="L157" s="4" t="inlineStr">
         <is>
           <t>Founder 2026-10-30</t>
         </is>

</xml_diff>